<commit_message>
Update runsetup_comact.xlsx fixture for testing
</commit_message>
<xml_diff>
--- a/tests/fixtures/wok_2026-07-07/runsetup_comact.xlsx
+++ b/tests/fixtures/wok_2026-07-07/runsetup_comact.xlsx
@@ -1867,7 +1867,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="111" customHeight="1" thickTop="1">
+    <row r="13" ht="48" customHeight="1" thickTop="1">
       <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Smyrna</t>
@@ -1929,24 +1929,18 @@
       </c>
       <c r="N13" s="88" t="inlineStr">
         <is>
-          <t>4/4 x RandomW x Sel 6 SEL OPT Unsel WOK
-4/4 x Rw &gt; 6 x RandomL +3" FAS OPT Unsel WOK
-4/4 x Rw SEL x RandomL +3" SEL OPT Unsel WOK
-4/4 x Rw &gt; 5 x RandomL +3" FAS OPT Unsel WOK
+          <t>4/4 x Rw &gt; 6 x RandomL +3" FAS OPT Unsel WOK
 4/4 x RandomW x RandomL +3" 3ACOM OPT Unsel WOK</t>
         </is>
       </c>
       <c r="O13" s="88" t="inlineStr">
         <is>
-          <t>16085783831819217
-17588035475183205
-25491
-25471
+          <t>17588035475183205
 25483</t>
         </is>
       </c>
       <c r="P13" s="89" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" ht="40.25" customHeight="1">
@@ -2049,7 +2043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="174" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="28" t="n"/>
       <c r="B16" s="29" t="n"/>
       <c r="C16" s="30" t="n"/>
@@ -2087,30 +2081,22 @@
       <c r="M16" s="33" t="n"/>
       <c r="N16" s="88" t="inlineStr">
         <is>
-          <t>4/4 x RandomW x Sel 6 SEL OPT Unsel WOK
-4/4 x RandomW x RandomL +3" 1COM OPT Unsel WOK
+          <t>4/4 x RandomW x RandomL +3" 1COM OPT Unsel WOK
 4/4 x RandomW x RandomL +3" 2COM OPT Unsel WOK
 4/4 x Rw &gt; 6 x RandomL +3" FAS OPT Unsel WOK
-4/4 x Rw &gt; 6 x RandomL +3" CHAR OPT ? WOK
-4/4 x Rw &gt; 8 x RandomL +3" CHAR OPT ? WOK
-4/4 x Rw SEL x RandomL +3" SEL OPT Unsel WOK
-4/4 x Rw &gt; 5 x RandomL +3" FAS OPT Unsel WOK</t>
+4/4 x Rw &gt; 6 x RandomL +3" CHAR OPT ? WOK</t>
         </is>
       </c>
       <c r="O16" s="88" t="inlineStr">
         <is>
-          <t>16085783831819217
-25475
+          <t>25475
 25479
 17588035475183205
-25487
-16195211180014552
-25491
-25471</t>
+25487</t>
         </is>
       </c>
       <c r="P16" s="89" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">

</xml_diff>